<commit_message>
alignment tools and minor updates
</commit_message>
<xml_diff>
--- a/Benchtop-CBI-Pittsburgh/parts-list/parts-list-immersion-cuvette.xlsx
+++ b/Benchtop-CBI-Pittsburgh/parts-list/parts-list-immersion-cuvette.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nikita\Documents\GitHub\mesoSPIM-bt-hardware\Benchtop-CBI-Pittsburgh\parts-list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74251AE3-39E3-498F-B524-34AEE61227E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EF93E86-AF55-4BFF-89C3-1C98093C240E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13692" yWindow="4224" windowWidth="24948" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5328" yWindow="4896" windowWidth="34560" windowHeight="18600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
   <si>
     <t xml:space="preserve">Part # </t>
   </si>
@@ -191,9 +191,6 @@
     <t>cuvette-v1.STL</t>
   </si>
   <si>
-    <t>Sealant: 10.1 oz Cartridge, Clear, Silicone</t>
-  </si>
-  <si>
     <t>Any similar consumer-grade silicone should do?</t>
   </si>
   <si>
@@ -201,6 +198,12 @@
   </si>
   <si>
     <t>https://brainresearchlab.com/product/adhesion-superfrost-plus-microscope-slides/</t>
+  </si>
+  <si>
+    <t>Red Devil Sealant: 10.1 oz Cartridge, Clear, Silicone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mscdirect.com/product/details/66239195 </t>
   </si>
 </sst>
 </file>
@@ -598,7 +601,7 @@
         <v>100</v>
       </c>
       <c r="G2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -676,7 +679,7 @@
         <v>164</v>
       </c>
       <c r="H5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -687,7 +690,7 @@
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -700,12 +703,16 @@
         <v>15</v>
       </c>
       <c r="G6" t="s">
-        <v>23</v>
+        <v>22</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="H3" r:id="rId1" xr:uid="{4394F167-51B7-4644-97D5-961D7C82B108}"/>
+    <hyperlink ref="H6" r:id="rId2" xr:uid="{B961D546-FD03-420D-A492-D7E5932E22DF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updates slide and sealant variants after successful tests
</commit_message>
<xml_diff>
--- a/Benchtop-CBI-Pittsburgh/parts-list/parts-list-immersion-cuvette.xlsx
+++ b/Benchtop-CBI-Pittsburgh/parts-list/parts-list-immersion-cuvette.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nikita\Documents\GitHub\mesoSPIM-bt-hardware\Benchtop-CBI-Pittsburgh\parts-list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EF93E86-AF55-4BFF-89C3-1C98093C240E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1D40D25-35FA-4BA0-A189-83E6968E71F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5328" yWindow="4896" windowWidth="34560" windowHeight="18600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7164" yWindow="7080" windowWidth="32100" windowHeight="16548" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
   <si>
     <t xml:space="preserve">Part # </t>
   </si>
@@ -66,9 +66,6 @@
   </si>
   <si>
     <t>varies</t>
-  </si>
-  <si>
-    <t>URL</t>
   </si>
   <si>
     <t>Amazon or AliExpress</t>
@@ -191,9 +188,6 @@
     <t>cuvette-v1.STL</t>
   </si>
   <si>
-    <t>Any similar consumer-grade silicone should do?</t>
-  </si>
-  <si>
     <t>Can be printed using Formlabs4 printer, suing Clear V5 Resin, with curing. CAD models in "...\custom_parts\ImmersionChambers\"</t>
   </si>
   <si>
@@ -204,6 +198,57 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.mscdirect.com/product/details/66239195 </t>
+  </si>
+  <si>
+    <t>Sealants that work well</t>
+  </si>
+  <si>
+    <t>SI595</t>
+  </si>
+  <si>
+    <t>Henkel</t>
+  </si>
+  <si>
+    <t>Loctite SI 595</t>
+  </si>
+  <si>
+    <t>Any similar consumer-grade silicone should do, but some are too viscous and hard to apply</t>
+  </si>
+  <si>
+    <t>Medium viscous, can be squuezed out with moderate force</t>
+  </si>
+  <si>
+    <t>https://www.henkel-adhesives.com/pa/en/product/flexible-sealants/loctite_si_595.html</t>
+  </si>
+  <si>
+    <t>249-75X50</t>
+  </si>
+  <si>
+    <t>Corning</t>
+  </si>
+  <si>
+    <t>https://ecatalog.corning.com/life-sciences/b2b/CH/en/General-Labware/Slides/Corning%C2%AE-Plain-Microscope-Slide/p/2947-75X50</t>
+  </si>
+  <si>
+    <t>https://www.fishersci.com/shop/products/plain-microscope-slides-15/125535B</t>
+  </si>
+  <si>
+    <t>URL1</t>
+  </si>
+  <si>
+    <t>URL2</t>
+  </si>
+  <si>
+    <t>Microscope slides that work well. Note their different width (38 or 50 mm), each requires a different chamber model</t>
+  </si>
+  <si>
+    <t>Microscope slides plain pre-cleaned 75x50x1 mm</t>
+  </si>
+  <si>
+    <t>Original slides used in CBI Pittsburgh</t>
+  </si>
+  <si>
+    <t>Modification (wide slides). Actual slide width is 51 mm, not 50. Come in huge box of 720 slides.</t>
   </si>
 </sst>
 </file>
@@ -235,12 +280,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -256,13 +307,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -544,17 +596,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.33203125" customWidth="1"/>
-    <col min="2" max="2" width="14.44140625" customWidth="1"/>
-    <col min="3" max="3" width="25.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.5546875" customWidth="1"/>
+    <col min="3" max="3" width="61.109375" customWidth="1"/>
     <col min="6" max="6" width="16.109375" customWidth="1"/>
     <col min="7" max="7" width="39.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -577,12 +629,15 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -601,18 +656,18 @@
         <v>100</v>
       </c>
       <c r="G2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
       <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
         <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
       </c>
       <c r="D3">
         <v>5</v>
@@ -621,25 +676,25 @@
         <v>20</v>
       </c>
       <c r="F3">
-        <f t="shared" ref="F3:F6" si="0">D3*E3</f>
+        <f t="shared" ref="F3:F9" si="0">D3*E3</f>
         <v>100</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -652,67 +707,132 @@
         <v>30</v>
       </c>
       <c r="G4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
         <v>17</v>
       </c>
-      <c r="H4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="C6" t="s">
         <v>19</v>
-      </c>
-      <c r="B5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>164</v>
-      </c>
-      <c r="F5">
-        <f t="shared" si="0"/>
-        <v>164</v>
-      </c>
-      <c r="H5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
-        <v>66239195</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" t="s">
-        <v>25</v>
       </c>
       <c r="D6">
         <v>1</v>
       </c>
       <c r="E6">
+        <v>164</v>
+      </c>
+      <c r="F6">
+        <f>D6*E6</f>
+        <v>164</v>
+      </c>
+      <c r="G6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>415</v>
+      </c>
+      <c r="G7" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" s="2">
+        <v>66239195</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
         <v>15</v>
       </c>
-      <c r="F6">
+      <c r="F9">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="G6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H6" s="3" t="s">
+      <c r="G9" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>26</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>25</v>
+      </c>
+      <c r="F10">
+        <v>25</v>
+      </c>
+      <c r="G10" t="s">
+        <v>30</v>
+      </c>
+      <c r="H10" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="H3" r:id="rId1" xr:uid="{4394F167-51B7-4644-97D5-961D7C82B108}"/>
-    <hyperlink ref="H6" r:id="rId2" xr:uid="{B961D546-FD03-420D-A492-D7E5932E22DF}"/>
+    <hyperlink ref="H9" r:id="rId2" xr:uid="{B961D546-FD03-420D-A492-D7E5932E22DF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
upload 50-mm wide window version (parts and photos)
</commit_message>
<xml_diff>
--- a/Benchtop-CBI-Pittsburgh/parts-list/parts-list-immersion-cuvette.xlsx
+++ b/Benchtop-CBI-Pittsburgh/parts-list/parts-list-immersion-cuvette.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nikita\Documents\GitHub\mesoSPIM-bt-hardware\Benchtop-CBI-Pittsburgh\parts-list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1D40D25-35FA-4BA0-A189-83E6968E71F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF323FA9-FD2C-46CD-A75E-C43784AA50C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7164" yWindow="7080" windowWidth="32100" windowHeight="16548" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10920" yWindow="4836" windowWidth="32100" windowHeight="16548" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="62">
   <si>
     <t xml:space="preserve">Part # </t>
   </si>
@@ -98,6 +98,134 @@
   </si>
   <si>
     <t>https://de.aliexpress.com/item/1005007537889780.html</t>
+  </si>
+  <si>
+    <t>https://de.aliexpress.com/item/1005001758039535.html</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Ulanzi U-100 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ball Head</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> for Tripod With Claw Quick Release Plate Mount</t>
+    </r>
+  </si>
+  <si>
+    <t>Brain Research Laboratories</t>
+  </si>
+  <si>
+    <t>3875-plus</t>
+  </si>
+  <si>
+    <t>38 x 75 x 1.0mm Adhesion Superfrost Plus (1 gross/144 slides)</t>
+  </si>
+  <si>
+    <t>cuvette-v1.STL</t>
+  </si>
+  <si>
+    <t>Can be printed using Formlabs4 printer, suing Clear V5 Resin, with curing. CAD models in "...\custom_parts\ImmersionChambers\"</t>
+  </si>
+  <si>
+    <t>https://brainresearchlab.com/product/adhesion-superfrost-plus-microscope-slides/</t>
+  </si>
+  <si>
+    <t>Red Devil Sealant: 10.1 oz Cartridge, Clear, Silicone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mscdirect.com/product/details/66239195 </t>
+  </si>
+  <si>
+    <t>SI595</t>
+  </si>
+  <si>
+    <t>Henkel</t>
+  </si>
+  <si>
+    <t>Loctite SI 595</t>
+  </si>
+  <si>
+    <t>Any similar consumer-grade silicone should do, but some are too viscous and hard to apply</t>
+  </si>
+  <si>
+    <t>https://www.henkel-adhesives.com/pa/en/product/flexible-sealants/loctite_si_595.html</t>
+  </si>
+  <si>
+    <t>249-75X50</t>
+  </si>
+  <si>
+    <t>Corning</t>
+  </si>
+  <si>
+    <t>https://ecatalog.corning.com/life-sciences/b2b/CH/en/General-Labware/Slides/Corning%C2%AE-Plain-Microscope-Slide/p/2947-75X50</t>
+  </si>
+  <si>
+    <t>https://www.fishersci.com/shop/products/plain-microscope-slides-15/125535B</t>
+  </si>
+  <si>
+    <t>URL1</t>
+  </si>
+  <si>
+    <t>URL2</t>
+  </si>
+  <si>
+    <t>Microscope slides plain pre-cleaned 75x50x1 mm</t>
+  </si>
+  <si>
+    <t>Original slides used in CBI Pittsburgh</t>
+  </si>
+  <si>
+    <t>Modification (wide slides). Actual slide width is 51 mm, not 50. Come in huge box of 720 slides.</t>
+  </si>
+  <si>
+    <t>cuvette-w70mm-slide50x75mm-v2.stp</t>
+  </si>
+  <si>
+    <t>SLS printed from PA12</t>
+  </si>
+  <si>
+    <t>cuvette frame, inner dimensions: 65x55x80mm</t>
+  </si>
+  <si>
+    <t>Larger cuvette than the original. CAD models in "...\custom_parts\ImmersionChambers\Slide-50x75mm-v1"</t>
+  </si>
+  <si>
+    <t>same as in the original</t>
+  </si>
+  <si>
+    <t>Medium viscous, can be squezed out with moderate force. Alternative to Red Devil, avaliable in Europe.</t>
+  </si>
+  <si>
+    <t>Tholabs</t>
+  </si>
+  <si>
+    <t>https://www.thorlabs.com/item/UBP2_M</t>
+  </si>
+  <si>
+    <t>UBP2/M</t>
+  </si>
+  <si>
+    <t>Universal Base Plate, 65 mm x 65 mm x 10 mm, Metric</t>
+  </si>
+  <si>
+    <t>Optional but nice to store cuvettes (wide base)</t>
   </si>
   <si>
     <r>
@@ -140,18 +268,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> (kit)</t>
-    </r>
-  </si>
-  <si>
-    <t>https://de.aliexpress.com/item/1005001758039535.html</t>
-  </si>
-  <si>
-    <t>Ulanzi U-100 Ball Head for Tripod With Claw Quick Release Plate Mount</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Ulanzi U-100 </t>
+      <t xml:space="preserve"> (</t>
     </r>
     <r>
       <rPr>
@@ -162,7 +279,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Ball Head</t>
+      <t>kit</t>
     </r>
     <r>
       <rPr>
@@ -172,90 +289,54 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> for Tripod With Claw Quick Release Plate Mount</t>
+      <t>)</t>
     </r>
   </si>
   <si>
-    <t>Brain Research Laboratories</t>
-  </si>
-  <si>
-    <t>3875-plus</t>
-  </si>
-  <si>
-    <t>38 x 75 x 1.0mm Adhesion Superfrost Plus (1 gross/144 slides)</t>
-  </si>
-  <si>
-    <t>cuvette-v1.STL</t>
-  </si>
-  <si>
-    <t>Can be printed using Formlabs4 printer, suing Clear V5 Resin, with curing. CAD models in "...\custom_parts\ImmersionChambers\"</t>
-  </si>
-  <si>
-    <t>https://brainresearchlab.com/product/adhesion-superfrost-plus-microscope-slides/</t>
-  </si>
-  <si>
-    <t>Red Devil Sealant: 10.1 oz Cartridge, Clear, Silicone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.mscdirect.com/product/details/66239195 </t>
-  </si>
-  <si>
-    <t>Sealants that work well</t>
-  </si>
-  <si>
-    <t>SI595</t>
-  </si>
-  <si>
-    <t>Henkel</t>
-  </si>
-  <si>
-    <t>Loctite SI 595</t>
-  </si>
-  <si>
-    <t>Any similar consumer-grade silicone should do, but some are too viscous and hard to apply</t>
-  </si>
-  <si>
-    <t>Medium viscous, can be squuezed out with moderate force</t>
-  </si>
-  <si>
-    <t>https://www.henkel-adhesives.com/pa/en/product/flexible-sealants/loctite_si_595.html</t>
-  </si>
-  <si>
-    <t>249-75X50</t>
-  </si>
-  <si>
-    <t>Corning</t>
-  </si>
-  <si>
-    <t>https://ecatalog.corning.com/life-sciences/b2b/CH/en/General-Labware/Slides/Corning%C2%AE-Plain-Microscope-Slide/p/2947-75X50</t>
-  </si>
-  <si>
-    <t>https://www.fishersci.com/shop/products/plain-microscope-slides-15/125535B</t>
-  </si>
-  <si>
-    <t>URL1</t>
-  </si>
-  <si>
-    <t>URL2</t>
-  </si>
-  <si>
-    <t>Microscope slides that work well. Note their different width (38 or 50 mm), each requires a different chamber model</t>
-  </si>
-  <si>
-    <t>Microscope slides plain pre-cleaned 75x50x1 mm</t>
-  </si>
-  <si>
-    <t>Original slides used in CBI Pittsburgh</t>
-  </si>
-  <si>
-    <t>Modification (wide slides). Actual slide width is 51 mm, not 50. Come in huge box of 720 slides.</t>
+    <t>Thorlabs</t>
+  </si>
+  <si>
+    <t>PS15M</t>
+  </si>
+  <si>
+    <t>Mounting Post Spacer, Height = 15 mm</t>
+  </si>
+  <si>
+    <t>https://www.thorlabs.com/item/PS15M</t>
+  </si>
+  <si>
+    <t>Pedestal</t>
+  </si>
+  <si>
+    <t>RC2/M</t>
+  </si>
+  <si>
+    <t>Dovetail Rail Carrier, 50.8 mm x 25.4 mm, M6 Counterbore, M4 Taps</t>
+  </si>
+  <si>
+    <t>https://www.thorlabs.com/item/RC2_M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1/4-20 socket head cap screw L=37 mm </t>
+  </si>
+  <si>
+    <t>Presentation: docs/Mesospim_cuvettes.pptx</t>
+  </si>
+  <si>
+    <t>Photos: docs/photos-version50mm-wide-SLSprinted(UZH)/</t>
+  </si>
+  <si>
+    <t>Modification (UZH): glass windows 50 mm wide</t>
+  </si>
+  <si>
+    <t>Original Version (CBI Pittsburgh): glass windows 38 mm wide</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -279,8 +360,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -289,7 +378,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -307,14 +402,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -596,10 +695,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" customWidth="1"/>
+    <col min="1" max="1" width="28.6640625" customWidth="1"/>
     <col min="2" max="2" width="23.5546875" customWidth="1"/>
     <col min="3" max="3" width="61.109375" customWidth="1"/>
     <col min="6" max="6" width="16.109375" customWidth="1"/>
@@ -629,45 +728,26 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2">
-        <v>5</v>
-      </c>
-      <c r="E2">
-        <v>20</v>
-      </c>
-      <c r="F2">
-        <f>D2*E2</f>
-        <v>100</v>
-      </c>
-      <c r="G2" t="s">
-        <v>21</v>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D3">
         <v>5</v>
@@ -676,14 +756,11 @@
         <v>20</v>
       </c>
       <c r="F3">
-        <f t="shared" ref="F3:F9" si="0">D3*E3</f>
+        <f>D3*E3</f>
         <v>100</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -694,39 +771,61 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>20</v>
+      </c>
+      <c r="F4">
+        <f t="shared" ref="F4:F7" si="0">D4*E4</f>
+        <v>100</v>
+      </c>
+      <c r="G4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5">
         <v>1</v>
       </c>
-      <c r="E4">
+      <c r="E5">
         <v>30</v>
       </c>
-      <c r="F4">
+      <c r="F5">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="G4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="G5" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
-        <v>38</v>
+      <c r="H5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
         <v>17</v>
-      </c>
-      <c r="C6" t="s">
-        <v>19</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -739,101 +838,263 @@
         <v>164</v>
       </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="H6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>32</v>
+      <c r="A7" s="2">
+        <v>66239195</v>
       </c>
       <c r="B7" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
+      <c r="E7">
+        <v>15</v>
+      </c>
       <c r="F7">
-        <v>415</v>
-      </c>
-      <c r="G7" t="s">
-        <v>41</v>
-      </c>
-      <c r="H7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I7" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
-        <v>66239195</v>
-      </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9">
-        <v>15</v>
-      </c>
-      <c r="F9">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G7" t="s">
+        <v>26</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12">
+        <v>5</v>
+      </c>
+      <c r="E12">
+        <v>50</v>
+      </c>
+      <c r="F12">
+        <f>D12*E12</f>
+        <v>250</v>
+      </c>
+      <c r="G12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13">
+        <v>5</v>
+      </c>
+      <c r="E13">
+        <v>20</v>
+      </c>
+      <c r="F13">
+        <f t="shared" ref="F13" si="1">D13*E13</f>
+        <v>100</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H13" s="3"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" t="s">
         <v>29</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="C14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>415</v>
+      </c>
+      <c r="F14">
+        <v>415</v>
+      </c>
+      <c r="G14" t="s">
+        <v>36</v>
+      </c>
+      <c r="H14" t="s">
+        <v>30</v>
+      </c>
+      <c r="I14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>25</v>
+      </c>
+      <c r="F15">
+        <v>25</v>
+      </c>
+      <c r="G15" t="s">
+        <v>42</v>
+      </c>
+      <c r="H15" t="s">
         <v>27</v>
       </c>
-      <c r="C10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10">
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16">
+        <v>5</v>
+      </c>
+      <c r="E16">
+        <v>41</v>
+      </c>
+      <c r="F16">
+        <f>D16*41</f>
+        <v>205</v>
+      </c>
+      <c r="G16" t="s">
+        <v>47</v>
+      </c>
+      <c r="H16" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17">
+        <v>2</v>
+      </c>
+      <c r="E17">
+        <v>11</v>
+      </c>
+      <c r="F17">
+        <f>D17*E17</f>
+        <v>22</v>
+      </c>
+      <c r="G17" t="s">
+        <v>53</v>
+      </c>
+      <c r="H17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" t="s">
+        <v>57</v>
+      </c>
+      <c r="D18">
         <v>1</v>
       </c>
-      <c r="E10">
-        <v>25</v>
-      </c>
-      <c r="F10">
-        <v>25</v>
-      </c>
-      <c r="G10" t="s">
-        <v>30</v>
-      </c>
-      <c r="H10" t="s">
-        <v>31</v>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18">
+        <f>D18*E18</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" t="s">
+        <v>55</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19">
+        <v>33</v>
+      </c>
+      <c r="F19">
+        <f>D19*E19</f>
+        <v>33</v>
+      </c>
+      <c r="H19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="7" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H3" r:id="rId1" xr:uid="{4394F167-51B7-4644-97D5-961D7C82B108}"/>
-    <hyperlink ref="H9" r:id="rId2" xr:uid="{B961D546-FD03-420D-A492-D7E5932E22DF}"/>
+    <hyperlink ref="H4" r:id="rId1" xr:uid="{4394F167-51B7-4644-97D5-961D7C82B108}"/>
+    <hyperlink ref="H7" r:id="rId2" xr:uid="{B961D546-FD03-420D-A492-D7E5932E22DF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>